<commit_message>
six MITRE ATT&CK in tables
</commit_message>
<xml_diff>
--- a/KandRStyle/research/MITREATTACK_Excel.xlsx
+++ b/KandRStyle/research/MITREATTACK_Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gladi\source\repos\bookWork2\KandRStyle\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9170C31B-AB5D-46F6-BBCC-FF1BAB81DF6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{734C0874-A107-4797-9EAC-F6BCD8C804FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14565" yWindow="-28920" windowWidth="16440" windowHeight="28320" activeTab="1" xr2:uid="{AAF9C8DB-DFC7-4AB7-B5CE-E4F6A7FEE475}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{AAF9C8DB-DFC7-4AB7-B5CE-E4F6A7FEE475}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="358">
   <si>
     <t>Create Account</t>
   </si>
@@ -1027,9 +1027,6 @@
     <t>Modify Cloud Compute Infrastructure  &amp;"Adversaries may create, modify, or delete cloud resources to achieve their objectives."\endnote{“Modify Cloud Compute Infrastructure, Technique T1578 - Enterprise | MITRE ATT\&amp;CK®." Mitre.Org, 2026, \url{https://attack.mitre.org/techniques/T1578/}. Accessed 13 July 2026.}\\</t>
   </si>
   <si>
-    <t>Modify Cloud Resource Hierarchy &amp;"Needs final verification"\endnote{“Modify Cloud Resource Hierarchy, Technique T1666 - Enterprise | MITRE ATT\&amp;CK®." Mitre.Org, 2026, \url{https://attack.mitre.org/techniques/T1666/}. Accessed 13 July 2026.}\\</t>
-  </si>
-  <si>
     <t>Modify Registry &amp;"Adversaries may interact with the Windows Registry to hide configuration information, modify system settings, or remove information as part of their attack."\endnote{“Modify Registry, Technique T1112 - Enterprise | MITRE ATT\&amp;CK®." Mitre.Org, 2026, \url{https://attack.mitre.org/techniques/T1112/}. Accessed 13 July 2026.}\\</t>
   </si>
   <si>
@@ -1112,6 +1109,12 @@
   </si>
   <si>
     <t>XSL Script Processing &amp;"Adversaries may bypass application control and obscure execution of code by embedding scripts inside XSL files."\endnote{“XSL Script Processing, Technique T1220 - Enterprise | MITRE ATT\&amp;CK®." Mitre.Org, 2026, \url{https://attack.mitre.org/techniques/T1220/}. Accessed 13 July 2026.}\\</t>
+  </si>
+  <si>
+    <t>Adversaries may attempt to modify hierarchical structures in infrastructure-as-a-service (IaaS) environments in order to evade defenses.</t>
+  </si>
+  <si>
+    <t>Modify Cloud Resource Hierarchy &amp;"Adversaries may attempt to modify hierarchical structures in infrastructure-as-a-service (IaaS) environments in order to evade defenses."\endnote{“Modify Cloud Resource Hierarchy, Technique T1666 - Enterprise | MITRE ATT\&amp;CK®." Mitre.Org, 2026, \url{https://attack.mitre.org/techniques/T1666/}. Accessed 13 July 2026.}\\</t>
   </si>
 </sst>
 </file>
@@ -4389,7 +4392,7 @@
         <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>328</v>
+        <v>357</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
@@ -4397,7 +4400,7 @@
         <v>33</v>
       </c>
       <c r="B37" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
@@ -4405,7 +4408,7 @@
         <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
@@ -4413,7 +4416,7 @@
         <v>35</v>
       </c>
       <c r="B39" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
@@ -4421,7 +4424,7 @@
         <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
@@ -4429,7 +4432,7 @@
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
@@ -4437,7 +4440,7 @@
         <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
@@ -4445,7 +4448,7 @@
         <v>39</v>
       </c>
       <c r="B43" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
@@ -4453,7 +4456,7 @@
         <v>40</v>
       </c>
       <c r="B44" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
@@ -4461,7 +4464,7 @@
         <v>41</v>
       </c>
       <c r="B45" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
@@ -4469,7 +4472,7 @@
         <v>42</v>
       </c>
       <c r="B46" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
@@ -4477,7 +4480,7 @@
         <v>43</v>
       </c>
       <c r="B47" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
@@ -4485,7 +4488,7 @@
         <v>44</v>
       </c>
       <c r="B48" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
@@ -4493,7 +4496,7 @@
         <v>45</v>
       </c>
       <c r="B49" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
@@ -4501,7 +4504,7 @@
         <v>46</v>
       </c>
       <c r="B50" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
@@ -4509,7 +4512,7 @@
         <v>47</v>
       </c>
       <c r="B51" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
@@ -4517,7 +4520,7 @@
         <v>48</v>
       </c>
       <c r="B52" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
@@ -4525,7 +4528,7 @@
         <v>49</v>
       </c>
       <c r="B53" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
@@ -4533,7 +4536,7 @@
         <v>50</v>
       </c>
       <c r="B54" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
@@ -4541,7 +4544,7 @@
         <v>51</v>
       </c>
       <c r="B55" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
@@ -4549,7 +4552,7 @@
         <v>52</v>
       </c>
       <c r="B56" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
@@ -4557,7 +4560,7 @@
         <v>53</v>
       </c>
       <c r="B57" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
@@ -4565,7 +4568,7 @@
         <v>54</v>
       </c>
       <c r="B58" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
@@ -4573,7 +4576,7 @@
         <v>55</v>
       </c>
       <c r="B59" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
@@ -4581,7 +4584,7 @@
         <v>56</v>
       </c>
       <c r="B60" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
@@ -4589,7 +4592,7 @@
         <v>57</v>
       </c>
       <c r="B61" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
@@ -4597,7 +4600,7 @@
         <v>58</v>
       </c>
       <c r="B62" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
@@ -4605,7 +4608,7 @@
         <v>59</v>
       </c>
       <c r="B63" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
@@ -4613,7 +4616,7 @@
         <v>60</v>
       </c>
       <c r="B64" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
   </sheetData>
@@ -5001,7 +5004,7 @@
         <v>96</v>
       </c>
       <c r="G32" t="s">
-        <v>200</v>
+        <v>356</v>
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.3">

</xml_diff>